<commit_message>
update lista de compras
</commit_message>
<xml_diff>
--- a/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
+++ b/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f391dd1b8209b4da/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\Trabajo Profesional de Ingeniería Electrónica\Tesis\docs\compras\Compra final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="8_{3D688A93-2F7E-4F93-B7F4-B6A61C18C032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C1DF20E-C942-465A-BEC4-29FE4DF998CC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A329FC31-DD14-4332-AEC1-A5BCE1359DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{725DC760-210F-4FF6-B798-3A0227CE396F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{725DC760-210F-4FF6-B798-3A0227CE396F}"/>
   </bookViews>
   <sheets>
     <sheet name="Materiales que faltan" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>ICL7660</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>2?</t>
   </si>
   <si>
     <t>1?</t>
@@ -111,7 +108,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,6 +253,13 @@
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -599,14 +603,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -617,51 +618,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -677,7 +684,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -993,20 +1000,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5053D558-D145-4D70-A7EA-6A3AE6B36176}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="44.28515625" customWidth="1"/>
     <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="6"/>
+    <col min="4" max="4" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -1023,11 +1030,11 @@
       <c r="B2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>14</v>
+      <c r="C2" s="4">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1037,10 +1044,10 @@
       <c r="B3" s="1">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1051,24 +1058,24 @@
       <c r="B4" s="1">
         <v>0</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="6">
         <v>0</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="8" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1079,16 +1086,16 @@
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>3</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
@@ -1096,7 +1103,7 @@
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>2</v>
       </c>
     </row>
@@ -1104,13 +1111,13 @@
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>22</v>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="C8" s="1">
         <v>4</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>5</v>
       </c>
     </row>
@@ -1118,13 +1125,13 @@
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="1">
         <v>1</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>10</v>
       </c>
     </row>
@@ -1138,7 +1145,7 @@
       <c r="C10" s="1">
         <v>1</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>2</v>
       </c>
     </row>
@@ -1152,7 +1159,7 @@
       <c r="C11" s="1">
         <v>1</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>3</v>
       </c>
     </row>
@@ -1166,7 +1173,7 @@
       <c r="C12" s="1">
         <v>1</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>4</v>
       </c>
     </row>
@@ -1177,43 +1184,40 @@
       <c r="B13" s="1">
         <v>1</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>19</v>
+      <c r="D13" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="1">
         <v>1</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>19</v>
+      <c r="C14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" s="1">
         <v>2</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <v>1</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
subida update lista de compras
</commit_message>
<xml_diff>
--- a/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
+++ b/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\Trabajo Profesional de Ingeniería Electrónica\Tesis\docs\compras\Compra final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A329FC31-DD14-4332-AEC1-A5BCE1359DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B68ECBEF-31AE-4BAC-B8DA-7469B3842893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{725DC760-210F-4FF6-B798-3A0227CE396F}"/>
   </bookViews>
@@ -603,7 +603,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -623,6 +623,10 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1108,44 +1112,44 @@
       </c>
     </row>
     <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="9">
         <v>4</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="9">
         <v>1</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="10">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="9">
         <v>1</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="9">
         <v>1</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="10">
         <v>2</v>
       </c>
     </row>
@@ -1157,10 +1161,10 @@
         <v>2</v>
       </c>
       <c r="C11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
conecta los gnd de la stm
</commit_message>
<xml_diff>
--- a/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
+++ b/docs/compras/Compra final/Lista de compras - Circuito Externo.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\Trabajo Profesional de Ingeniería Electrónica\Tesis\docs\compras\Compra final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\---\Desktop\Tesis\docs\compras\Compra final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B68ECBEF-31AE-4BAC-B8DA-7469B3842893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{725DC760-210F-4FF6-B798-3A0227CE396F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Materiales que faltan" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>ICL7660</t>
   </si>
@@ -55,9 +55,6 @@
     <t>DIP switch de 1</t>
   </si>
   <si>
-    <t>Sensor de corriente (INA180 o AD620)</t>
-  </si>
-  <si>
     <t>R 33kΩ</t>
   </si>
   <si>
@@ -76,23 +73,20 @@
     <t>Total</t>
   </si>
   <si>
-    <t>1?</t>
-  </si>
-  <si>
     <t>IRLB8721 (N-MOSFET de celda)</t>
   </si>
   <si>
-    <t>0?</t>
-  </si>
-  <si>
     <t>0 (1 del central +1 del 4to banco - 3 que tenemos)</t>
   </si>
   <si>
     <t>MMBFJ201 (JFET para los bancos)</t>
   </si>
   <si>
+    <t>Sensor de corriente (INA180)</t>
+  </si>
+  <si>
     <r>
-      <t>R shunt 2512 1m</t>
+      <t>R shunt 2512 50m</t>
     </r>
     <r>
       <rPr>
@@ -103,12 +97,49 @@
       <t>Ω</t>
     </r>
   </si>
+  <si>
+    <t>Quad-opamp TL084:</t>
+  </si>
+  <si>
+    <t>Conectores cable plano macho 2x7:</t>
+  </si>
+  <si>
+    <t>Capacitores 100nF:</t>
+  </si>
+  <si>
+    <t>DIP switch de 4 posiciones:</t>
+  </si>
+  <si>
+    <t>DIP switch de 1 posicion:</t>
+  </si>
+  <si>
+    <t>Sensor de corriente (INA180):</t>
+  </si>
+  <si>
+    <t>IRLB8721:</t>
+  </si>
+  <si>
+    <t>MMBFJ201 :</t>
+  </si>
+  <si>
+    <r>
+      <t>R shunt 2512 50m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ω 1W:</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -631,48 +662,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Buena" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1003,31 +1034,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5053D558-D145-4D70-A7EA-6A3AE6B36176}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="44.28515625" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="5"/>
+    <col min="2" max="2" width="44.25" customWidth="1"/>
+    <col min="3" max="3" width="31.375" customWidth="1"/>
+    <col min="4" max="4" width="11.375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="30">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1041,35 +1072,35 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" s="1" customFormat="1">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="6" customFormat="1">
+      <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="6">
         <v>0</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="6" customFormat="1">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1080,26 +1111,26 @@
         <v>6</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="1" customFormat="1">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="4">
         <v>3</v>
       </c>
       <c r="D6" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1">
         <v>1</v>
@@ -1111,12 +1142,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" s="1" customFormat="1">
       <c r="A8" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C8" s="9">
         <v>4</v>
@@ -1125,12 +1156,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" s="1" customFormat="1">
       <c r="A9" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="9">
         <v>1</v>
@@ -1139,7 +1170,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" s="1" customFormat="1">
       <c r="A10" s="9" t="s">
         <v>8</v>
       </c>
@@ -1153,7 +1184,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" s="1" customFormat="1">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1167,7 +1198,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" s="1" customFormat="1">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1175,43 +1206,43 @@
         <v>3</v>
       </c>
       <c r="C12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="1" customFormat="1">
       <c r="A13" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B13" s="1">
-        <v>1</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" s="1" customFormat="1">
       <c r="A14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B14" s="1">
-        <v>1</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="B15" s="1">
         <v>2</v>
@@ -1227,4 +1258,98 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="5">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>